<commit_message>
feat(pipeline): complete 7-step strong-gating flow for tran_cdm_dim_cstm_dmns_h.sql
</commit_message>
<xml_diff>
--- a/Version/BATCH/ETL/APP/CDM/BIN/tran_cdm_dim_cstm_dmns_h.xlsx
+++ b/Version/BATCH/ETL/APP/CDM/BIN/tran_cdm_dim_cstm_dmns_h.xlsx
@@ -598,22 +598,22 @@
     <t>N</t>
   </si>
   <si>
+    <t>未添加企业微信</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
     <t>UNKN_</t>
   </si>
   <si>
     <t>365</t>
   </si>
   <si>
-    <t>未添加企业微信</t>
-  </si>
-  <si>
-    <t>Y</t>
+    <t>18</t>
   </si>
   <si>
     <t>1+0</t>
-  </si>
-  <si>
-    <t>18</t>
   </si>
   <si>
     <t>来源系统名</t>
@@ -11274,7 +11274,7 @@
         <v>35</v>
       </c>
       <c r="E27" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="F27" t="s">
         <v>189</v>
@@ -11288,19 +11288,19 @@
     <row r="28">
       <c r="A28"/>
       <c r="B28" t="s">
-        <v>10</v>
+        <v>86</v>
       </c>
       <c r="C28" t="s">
-        <v>11</v>
+        <v>113</v>
       </c>
       <c r="D28" t="s">
-        <v>35</v>
+        <v>133</v>
       </c>
       <c r="E28" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="F28" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="G28" t="s">
         <v>149</v>
@@ -11317,7 +11317,7 @@
         <v>11</v>
       </c>
       <c r="D29" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="E29" t="s">
         <v>188</v>
@@ -11334,19 +11334,19 @@
     <row r="30">
       <c r="A30"/>
       <c r="B30" t="s">
-        <v>86</v>
+        <v>10</v>
       </c>
       <c r="C30" t="s">
-        <v>113</v>
+        <v>11</v>
       </c>
       <c r="D30" t="s">
-        <v>133</v>
+        <v>24</v>
       </c>
       <c r="E30" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F30" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="G30" t="s">
         <v>149</v>
@@ -11409,7 +11409,7 @@
         <v>11</v>
       </c>
       <c r="D33" t="s">
-        <v>67</v>
+        <v>35</v>
       </c>
       <c r="E33" t="s">
         <v>193</v>
@@ -11432,7 +11432,7 @@
         <v>11</v>
       </c>
       <c r="D34" t="s">
-        <v>35</v>
+        <v>67</v>
       </c>
       <c r="E34" t="s">
         <v>193</v>
@@ -11455,10 +11455,10 @@
         <v>11</v>
       </c>
       <c r="D35" t="s">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="E35" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="F35" t="s">
         <v>189</v>
@@ -11478,10 +11478,10 @@
         <v>11</v>
       </c>
       <c r="D36" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="E36" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F36" t="s">
         <v>189</v>
@@ -11501,10 +11501,10 @@
         <v>11</v>
       </c>
       <c r="D37" t="s">
-        <v>76</v>
+        <v>13</v>
       </c>
       <c r="E37" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="F37" t="s">
         <v>189</v>
@@ -11524,10 +11524,10 @@
         <v>11</v>
       </c>
       <c r="D38" t="s">
-        <v>16</v>
+        <v>48</v>
       </c>
       <c r="E38" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F38" t="s">
         <v>189</v>
@@ -11547,7 +11547,7 @@
         <v>11</v>
       </c>
       <c r="D39" t="s">
-        <v>13</v>
+        <v>35</v>
       </c>
       <c r="E39" t="s">
         <v>195</v>
@@ -11570,10 +11570,10 @@
         <v>11</v>
       </c>
       <c r="D40" t="s">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="E40" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="F40" t="s">
         <v>189</v>
@@ -11593,10 +11593,10 @@
         <v>11</v>
       </c>
       <c r="D41" t="s">
-        <v>48</v>
+        <v>13</v>
       </c>
       <c r="E41" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F41" t="s">
         <v>189</v>
@@ -11619,7 +11619,7 @@
         <v>35</v>
       </c>
       <c r="E42" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="F42" t="s">
         <v>189</v>
@@ -11639,10 +11639,10 @@
         <v>11</v>
       </c>
       <c r="D43" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E43" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="F43" t="s">
         <v>189</v>
@@ -11665,7 +11665,7 @@
         <v>67</v>
       </c>
       <c r="E44" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="F44" t="s">
         <v>189</v>
@@ -11685,10 +11685,10 @@
         <v>11</v>
       </c>
       <c r="D45" t="s">
-        <v>13</v>
+        <v>35</v>
       </c>
       <c r="E45" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="F45" t="s">
         <v>189</v>
@@ -11708,10 +11708,10 @@
         <v>11</v>
       </c>
       <c r="D46" t="s">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="E46" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="F46" t="s">
         <v>189</v>
@@ -11731,7 +11731,7 @@
         <v>11</v>
       </c>
       <c r="D47" t="s">
-        <v>43</v>
+        <v>13</v>
       </c>
       <c r="E47" t="s">
         <v>193</v>
@@ -11777,10 +11777,10 @@
         <v>11</v>
       </c>
       <c r="D49" t="s">
-        <v>16</v>
+        <v>68</v>
       </c>
       <c r="E49" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F49" t="s">
         <v>189</v>
@@ -11800,10 +11800,10 @@
         <v>11</v>
       </c>
       <c r="D50" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="E50" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F50" t="s">
         <v>189</v>
@@ -11823,10 +11823,10 @@
         <v>11</v>
       </c>
       <c r="D51" t="s">
-        <v>76</v>
+        <v>16</v>
       </c>
       <c r="E51" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="F51" t="s">
         <v>189</v>
@@ -11849,7 +11849,7 @@
         <v>43</v>
       </c>
       <c r="E52" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="F52" t="s">
         <v>189</v>
@@ -11869,10 +11869,10 @@
         <v>11</v>
       </c>
       <c r="D53" t="s">
-        <v>54</v>
+        <v>81</v>
       </c>
       <c r="E53" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="F53" t="s">
         <v>189</v>
@@ -11892,10 +11892,10 @@
         <v>11</v>
       </c>
       <c r="D54" t="s">
-        <v>81</v>
+        <v>55</v>
       </c>
       <c r="E54" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="F54" t="s">
         <v>189</v>
@@ -11915,10 +11915,10 @@
         <v>11</v>
       </c>
       <c r="D55" t="s">
-        <v>74</v>
+        <v>32</v>
       </c>
       <c r="E55" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="F55" t="s">
         <v>189</v>
@@ -11938,10 +11938,10 @@
         <v>11</v>
       </c>
       <c r="D56" t="s">
-        <v>32</v>
+        <v>74</v>
       </c>
       <c r="E56" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="F56" t="s">
         <v>189</v>
@@ -11961,10 +11961,10 @@
         <v>11</v>
       </c>
       <c r="D57" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E57" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="F57" t="s">
         <v>189</v>
@@ -11987,13 +11987,13 @@
         <v>93</v>
       </c>
       <c r="E58" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="F58" t="s">
         <v>182</v>
       </c>
       <c r="G58" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="H58"/>
       <c r="I58"/>
@@ -12004,19 +12004,19 @@
         <v>10</v>
       </c>
       <c r="C59" t="s">
-        <v>90</v>
+        <v>11</v>
       </c>
       <c r="D59" t="s">
-        <v>93</v>
+        <v>75</v>
       </c>
       <c r="E59" t="s">
         <v>185</v>
       </c>
       <c r="F59" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="G59" t="s">
-        <v>21</v>
+        <v>149</v>
       </c>
       <c r="H59"/>
       <c r="I59"/>
@@ -12024,13 +12024,13 @@
     <row r="60">
       <c r="A60"/>
       <c r="B60" t="s">
-        <v>86</v>
+        <v>10</v>
       </c>
       <c r="C60" t="s">
-        <v>113</v>
+        <v>90</v>
       </c>
       <c r="D60" t="s">
-        <v>133</v>
+        <v>93</v>
       </c>
       <c r="E60" t="s">
         <v>185</v>
@@ -12039,7 +12039,7 @@
         <v>182</v>
       </c>
       <c r="G60" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="H60"/>
       <c r="I60"/>
@@ -12047,13 +12047,13 @@
     <row r="61">
       <c r="A61"/>
       <c r="B61" t="s">
-        <v>86</v>
+        <v>10</v>
       </c>
       <c r="C61" t="s">
-        <v>113</v>
+        <v>90</v>
       </c>
       <c r="D61" t="s">
-        <v>133</v>
+        <v>93</v>
       </c>
       <c r="E61" t="s">
         <v>185</v>
@@ -12062,7 +12062,7 @@
         <v>182</v>
       </c>
       <c r="G61" t="s">
-        <v>79</v>
+        <v>55</v>
       </c>
       <c r="H61"/>
       <c r="I61"/>
@@ -12073,19 +12073,19 @@
         <v>10</v>
       </c>
       <c r="C62" t="s">
-        <v>90</v>
+        <v>11</v>
       </c>
       <c r="D62" t="s">
-        <v>93</v>
+        <v>23</v>
       </c>
       <c r="E62" t="s">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="F62" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="G62" t="s">
-        <v>79</v>
+        <v>149</v>
       </c>
       <c r="H62"/>
       <c r="I62"/>
@@ -12099,16 +12099,16 @@
         <v>113</v>
       </c>
       <c r="D63" t="s">
-        <v>133</v>
+        <v>142</v>
       </c>
       <c r="E63" t="s">
-        <v>185</v>
+        <v>198</v>
       </c>
       <c r="F63" t="s">
         <v>182</v>
       </c>
       <c r="G63" t="s">
-        <v>27</v>
+        <v>75</v>
       </c>
       <c r="H63"/>
       <c r="I63"/>
@@ -12116,22 +12116,22 @@
     <row r="64">
       <c r="A64"/>
       <c r="B64" t="s">
-        <v>10</v>
+        <v>86</v>
       </c>
       <c r="C64" t="s">
-        <v>11</v>
+        <v>113</v>
       </c>
       <c r="D64" t="s">
-        <v>72</v>
+        <v>133</v>
       </c>
       <c r="E64" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="F64" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="G64" t="s">
-        <v>149</v>
+        <v>85</v>
       </c>
       <c r="H64"/>
       <c r="I64"/>
@@ -12142,19 +12142,19 @@
         <v>10</v>
       </c>
       <c r="C65" t="s">
-        <v>11</v>
+        <v>90</v>
       </c>
       <c r="D65" t="s">
-        <v>35</v>
+        <v>93</v>
       </c>
       <c r="E65" t="s">
         <v>185</v>
       </c>
       <c r="F65" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="G65" t="s">
-        <v>149</v>
+        <v>27</v>
       </c>
       <c r="H65"/>
       <c r="I65"/>
@@ -12162,13 +12162,13 @@
     <row r="66">
       <c r="A66"/>
       <c r="B66" t="s">
-        <v>86</v>
+        <v>10</v>
       </c>
       <c r="C66" t="s">
-        <v>113</v>
+        <v>90</v>
       </c>
       <c r="D66" t="s">
-        <v>133</v>
+        <v>93</v>
       </c>
       <c r="E66" t="s">
         <v>185</v>
@@ -12185,13 +12185,13 @@
     <row r="67">
       <c r="A67"/>
       <c r="B67" t="s">
-        <v>10</v>
+        <v>86</v>
       </c>
       <c r="C67" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="D67" t="s">
-        <v>93</v>
+        <v>133</v>
       </c>
       <c r="E67" t="s">
         <v>185</v>
@@ -12200,7 +12200,7 @@
         <v>182</v>
       </c>
       <c r="G67" t="s">
-        <v>74</v>
+        <v>54</v>
       </c>
       <c r="H67"/>
       <c r="I67"/>
@@ -12217,13 +12217,13 @@
         <v>133</v>
       </c>
       <c r="E68" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="F68" t="s">
         <v>182</v>
       </c>
       <c r="G68" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="H68"/>
       <c r="I68"/>
@@ -12231,22 +12231,22 @@
     <row r="69">
       <c r="A69"/>
       <c r="B69" t="s">
-        <v>86</v>
+        <v>10</v>
       </c>
       <c r="C69" t="s">
-        <v>113</v>
+        <v>11</v>
       </c>
       <c r="D69" t="s">
-        <v>133</v>
+        <v>12</v>
       </c>
       <c r="E69" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F69" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="G69" t="s">
-        <v>35</v>
+        <v>149</v>
       </c>
       <c r="H69"/>
       <c r="I69"/>
@@ -12263,13 +12263,13 @@
         <v>133</v>
       </c>
       <c r="E70" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="F70" t="s">
         <v>182</v>
       </c>
       <c r="G70" t="s">
-        <v>35</v>
+        <v>79</v>
       </c>
       <c r="H70"/>
       <c r="I70"/>
@@ -12277,13 +12277,13 @@
     <row r="71">
       <c r="A71"/>
       <c r="B71" t="s">
-        <v>10</v>
+        <v>86</v>
       </c>
       <c r="C71" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="D71" t="s">
-        <v>93</v>
+        <v>133</v>
       </c>
       <c r="E71" t="s">
         <v>185</v>
@@ -12292,7 +12292,7 @@
         <v>182</v>
       </c>
       <c r="G71" t="s">
-        <v>35</v>
+        <v>81</v>
       </c>
       <c r="H71"/>
       <c r="I71"/>
@@ -12300,13 +12300,13 @@
     <row r="72">
       <c r="A72"/>
       <c r="B72" t="s">
-        <v>10</v>
+        <v>86</v>
       </c>
       <c r="C72" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="D72" t="s">
-        <v>93</v>
+        <v>133</v>
       </c>
       <c r="E72" t="s">
         <v>190</v>
@@ -12315,7 +12315,7 @@
         <v>182</v>
       </c>
       <c r="G72" t="s">
-        <v>68</v>
+        <v>37</v>
       </c>
       <c r="H72"/>
       <c r="I72"/>
@@ -12326,19 +12326,19 @@
         <v>10</v>
       </c>
       <c r="C73" t="s">
-        <v>90</v>
+        <v>11</v>
       </c>
       <c r="D73" t="s">
-        <v>93</v>
+        <v>12</v>
       </c>
       <c r="E73" t="s">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="F73" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="G73" t="s">
-        <v>81</v>
+        <v>149</v>
       </c>
       <c r="H73"/>
       <c r="I73"/>
@@ -12361,7 +12361,7 @@
         <v>182</v>
       </c>
       <c r="G74" t="s">
-        <v>81</v>
+        <v>35</v>
       </c>
       <c r="H74"/>
       <c r="I74"/>
@@ -12369,22 +12369,22 @@
     <row r="75">
       <c r="A75"/>
       <c r="B75" t="s">
-        <v>86</v>
+        <v>10</v>
       </c>
       <c r="C75" t="s">
-        <v>113</v>
+        <v>90</v>
       </c>
       <c r="D75" t="s">
-        <v>133</v>
+        <v>93</v>
       </c>
       <c r="E75" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="F75" t="s">
         <v>182</v>
       </c>
       <c r="G75" t="s">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="H75"/>
       <c r="I75"/>
@@ -12398,10 +12398,10 @@
         <v>11</v>
       </c>
       <c r="D76" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="E76" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F76" t="s">
         <v>189</v>
@@ -12415,13 +12415,13 @@
     <row r="77">
       <c r="A77"/>
       <c r="B77" t="s">
-        <v>10</v>
+        <v>86</v>
       </c>
       <c r="C77" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="D77" t="s">
-        <v>93</v>
+        <v>133</v>
       </c>
       <c r="E77" t="s">
         <v>190</v>
@@ -12430,7 +12430,7 @@
         <v>182</v>
       </c>
       <c r="G77" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H77"/>
       <c r="I77"/>
@@ -12438,22 +12438,22 @@
     <row r="78">
       <c r="A78"/>
       <c r="B78" t="s">
-        <v>10</v>
+        <v>86</v>
       </c>
       <c r="C78" t="s">
-        <v>11</v>
+        <v>113</v>
       </c>
       <c r="D78" t="s">
-        <v>23</v>
+        <v>133</v>
       </c>
       <c r="E78" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="F78" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="G78" t="s">
-        <v>149</v>
+        <v>74</v>
       </c>
       <c r="H78"/>
       <c r="I78"/>
@@ -12461,22 +12461,22 @@
     <row r="79">
       <c r="A79"/>
       <c r="B79" t="s">
-        <v>86</v>
+        <v>10</v>
       </c>
       <c r="C79" t="s">
-        <v>113</v>
+        <v>90</v>
       </c>
       <c r="D79" t="s">
-        <v>133</v>
+        <v>93</v>
       </c>
       <c r="E79" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="F79" t="s">
         <v>182</v>
       </c>
       <c r="G79" t="s">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="H79"/>
       <c r="I79"/>
@@ -12487,19 +12487,19 @@
         <v>10</v>
       </c>
       <c r="C80" t="s">
-        <v>90</v>
+        <v>11</v>
       </c>
       <c r="D80" t="s">
-        <v>93</v>
+        <v>39</v>
       </c>
       <c r="E80" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="F80" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="G80" t="s">
-        <v>35</v>
+        <v>149</v>
       </c>
       <c r="H80"/>
       <c r="I80"/>
@@ -12507,22 +12507,22 @@
     <row r="81">
       <c r="A81"/>
       <c r="B81" t="s">
-        <v>86</v>
+        <v>10</v>
       </c>
       <c r="C81" t="s">
-        <v>113</v>
+        <v>90</v>
       </c>
       <c r="D81" t="s">
-        <v>133</v>
+        <v>93</v>
       </c>
       <c r="E81" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="F81" t="s">
         <v>182</v>
       </c>
       <c r="G81" t="s">
-        <v>21</v>
+        <v>68</v>
       </c>
       <c r="H81"/>
       <c r="I81"/>
@@ -12530,22 +12530,22 @@
     <row r="82">
       <c r="A82"/>
       <c r="B82" t="s">
-        <v>10</v>
+        <v>86</v>
       </c>
       <c r="C82" t="s">
-        <v>11</v>
+        <v>113</v>
       </c>
       <c r="D82" t="s">
-        <v>75</v>
+        <v>142</v>
       </c>
       <c r="E82" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="F82" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="G82" t="s">
-        <v>149</v>
+        <v>35</v>
       </c>
       <c r="H82"/>
       <c r="I82"/>
@@ -12556,19 +12556,19 @@
         <v>10</v>
       </c>
       <c r="C83" t="s">
-        <v>11</v>
+        <v>90</v>
       </c>
       <c r="D83" t="s">
-        <v>73</v>
+        <v>93</v>
       </c>
       <c r="E83" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="F83" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="G83" t="s">
-        <v>149</v>
+        <v>75</v>
       </c>
       <c r="H83"/>
       <c r="I83"/>
@@ -12576,13 +12576,13 @@
     <row r="84">
       <c r="A84"/>
       <c r="B84" t="s">
-        <v>10</v>
+        <v>86</v>
       </c>
       <c r="C84" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="D84" t="s">
-        <v>93</v>
+        <v>142</v>
       </c>
       <c r="E84" t="s">
         <v>198</v>
@@ -12591,7 +12591,7 @@
         <v>182</v>
       </c>
       <c r="G84" t="s">
-        <v>75</v>
+        <v>35</v>
       </c>
       <c r="H84"/>
       <c r="I84"/>
@@ -12605,10 +12605,10 @@
         <v>11</v>
       </c>
       <c r="D85" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="E85" t="s">
-        <v>186</v>
+        <v>196</v>
       </c>
       <c r="F85" t="s">
         <v>189</v>
@@ -12622,22 +12622,22 @@
     <row r="86">
       <c r="A86"/>
       <c r="B86" t="s">
-        <v>86</v>
+        <v>10</v>
       </c>
       <c r="C86" t="s">
-        <v>113</v>
+        <v>11</v>
       </c>
       <c r="D86" t="s">
-        <v>142</v>
+        <v>83</v>
       </c>
       <c r="E86" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F86" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="G86" t="s">
-        <v>35</v>
+        <v>149</v>
       </c>
       <c r="H86"/>
       <c r="I86"/>
@@ -12651,16 +12651,16 @@
         <v>113</v>
       </c>
       <c r="D87" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="E87" t="s">
-        <v>199</v>
+        <v>185</v>
       </c>
       <c r="F87" t="s">
         <v>182</v>
       </c>
       <c r="G87" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="H87"/>
       <c r="I87"/>
@@ -12671,19 +12671,19 @@
         <v>10</v>
       </c>
       <c r="C88" t="s">
-        <v>11</v>
+        <v>90</v>
       </c>
       <c r="D88" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="E88" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="F88" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="G88" t="s">
-        <v>149</v>
+        <v>35</v>
       </c>
       <c r="H88"/>
       <c r="I88"/>
@@ -12694,19 +12694,19 @@
         <v>10</v>
       </c>
       <c r="C89" t="s">
-        <v>11</v>
+        <v>90</v>
       </c>
       <c r="D89" t="s">
-        <v>12</v>
+        <v>93</v>
       </c>
       <c r="E89" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="F89" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="G89" t="s">
-        <v>149</v>
+        <v>35</v>
       </c>
       <c r="H89"/>
       <c r="I89"/>
@@ -12714,22 +12714,22 @@
     <row r="90">
       <c r="A90"/>
       <c r="B90" t="s">
-        <v>10</v>
+        <v>86</v>
       </c>
       <c r="C90" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="D90" t="s">
-        <v>93</v>
+        <v>142</v>
       </c>
       <c r="E90" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="F90" t="s">
         <v>182</v>
       </c>
       <c r="G90" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="H90"/>
       <c r="I90"/>
@@ -12752,7 +12752,7 @@
         <v>182</v>
       </c>
       <c r="G91" t="s">
-        <v>54</v>
+        <v>21</v>
       </c>
       <c r="H91"/>
       <c r="I91"/>
@@ -12763,19 +12763,19 @@
         <v>10</v>
       </c>
       <c r="C92" t="s">
-        <v>11</v>
+        <v>90</v>
       </c>
       <c r="D92" t="s">
-        <v>39</v>
+        <v>93</v>
       </c>
       <c r="E92" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="F92" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="G92" t="s">
-        <v>149</v>
+        <v>35</v>
       </c>
       <c r="H92"/>
       <c r="I92"/>
@@ -12789,16 +12789,16 @@
         <v>113</v>
       </c>
       <c r="D93" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="E93" t="s">
-        <v>199</v>
+        <v>185</v>
       </c>
       <c r="F93" t="s">
         <v>182</v>
       </c>
       <c r="G93" t="s">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="H93"/>
       <c r="I93"/>
@@ -12806,22 +12806,22 @@
     <row r="94">
       <c r="A94"/>
       <c r="B94" t="s">
-        <v>86</v>
+        <v>10</v>
       </c>
       <c r="C94" t="s">
-        <v>113</v>
+        <v>11</v>
       </c>
       <c r="D94" t="s">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="E94" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
       <c r="F94" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="G94" t="s">
-        <v>75</v>
+        <v>149</v>
       </c>
       <c r="H94"/>
       <c r="I94"/>
@@ -12838,13 +12838,13 @@
         <v>93</v>
       </c>
       <c r="E95" t="s">
-        <v>198</v>
+        <v>185</v>
       </c>
       <c r="F95" t="s">
         <v>182</v>
       </c>
       <c r="G95" t="s">
-        <v>35</v>
+        <v>85</v>
       </c>
       <c r="H95"/>
       <c r="I95"/>
@@ -12852,13 +12852,13 @@
     <row r="96">
       <c r="A96"/>
       <c r="B96" t="s">
-        <v>10</v>
+        <v>86</v>
       </c>
       <c r="C96" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="D96" t="s">
-        <v>93</v>
+        <v>133</v>
       </c>
       <c r="E96" t="s">
         <v>185</v>
@@ -12875,22 +12875,22 @@
     <row r="97">
       <c r="A97"/>
       <c r="B97" t="s">
-        <v>86</v>
+        <v>10</v>
       </c>
       <c r="C97" t="s">
-        <v>113</v>
+        <v>11</v>
       </c>
       <c r="D97" t="s">
-        <v>133</v>
+        <v>83</v>
       </c>
       <c r="E97" t="s">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="F97" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="G97" t="s">
-        <v>54</v>
+        <v>149</v>
       </c>
       <c r="H97"/>
       <c r="I97"/>

</xml_diff>